<commit_message>
Marked all entries removed where the date is before next release
</commit_message>
<xml_diff>
--- a/work-in-progress/Peppol Code Lists - Document types v9.6.xlsx
+++ b/work-in-progress/Peppol Code Lists - Document types v9.6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\git-peppol\peppol-edec-codelists\work-in-progress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65013164-8BF7-4570-81E5-835CCDC5D5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D336D0A-29A8-4BDE-9D2A-63FBDADA6525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="135" yWindow="720" windowWidth="25875" windowHeight="20160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2911,7 +2911,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3037,11 +3037,6 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -5334,89 +5329,89 @@
         <v>123</v>
       </c>
     </row>
-    <row r="47" spans="1:14" s="31" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A47" s="31" t="s">
+    <row r="47" spans="1:14" s="13" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A47" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B47" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C47" s="31" t="s">
+      <c r="B47" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="D47" s="28">
+      <c r="D47" s="25">
         <v>3</v>
       </c>
-      <c r="E47" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F47" s="33" t="s">
+      <c r="E47" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F47" s="15" t="s">
         <v>825</v>
       </c>
-      <c r="G47" s="42">
+      <c r="G47" s="44">
         <v>46025</v>
       </c>
-      <c r="H47" s="31" t="s">
+      <c r="H47" s="13" t="s">
         <v>826</v>
       </c>
-      <c r="I47" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J47" s="31" t="b">
+      <c r="I47" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J47" s="13" t="b">
         <f>FALSE</f>
         <v>0</v>
       </c>
-      <c r="K47" s="29"/>
-      <c r="L47" s="27" t="s">
+      <c r="K47" s="21"/>
+      <c r="L47" s="14" t="s">
         <v>555</v>
       </c>
-      <c r="M47" s="27" t="s">
+      <c r="M47" s="14" t="s">
         <v>673</v>
       </c>
-      <c r="N47" s="31" t="s">
+      <c r="N47" s="16" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="48" spans="1:14" s="31" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A48" s="31" t="s">
+    <row r="48" spans="1:14" s="13" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A48" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B48" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C48" s="31" t="s">
+      <c r="B48" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C48" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="D48" s="28">
+      <c r="D48" s="25">
         <v>3</v>
       </c>
-      <c r="E48" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F48" s="33" t="s">
+      <c r="E48" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F48" s="15" t="s">
         <v>825</v>
       </c>
-      <c r="G48" s="42">
+      <c r="G48" s="44">
         <v>46025</v>
       </c>
-      <c r="H48" s="31" t="s">
+      <c r="H48" s="13" t="s">
         <v>826</v>
       </c>
-      <c r="I48" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J48" s="31" t="b">
+      <c r="I48" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J48" s="13" t="b">
         <f>FALSE</f>
         <v>0</v>
       </c>
-      <c r="K48" s="29"/>
-      <c r="L48" s="27" t="s">
+      <c r="K48" s="21"/>
+      <c r="L48" s="14" t="s">
         <v>555</v>
       </c>
-      <c r="M48" s="27" t="s">
+      <c r="M48" s="14" t="s">
         <v>674</v>
       </c>
-      <c r="N48" s="31" t="s">
+      <c r="N48" s="16" t="s">
         <v>122</v>
       </c>
     </row>
@@ -6297,179 +6292,179 @@
         <v>134</v>
       </c>
     </row>
-    <row r="72" spans="1:14" s="31" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A72" s="31" t="s">
+    <row r="72" spans="1:14" s="13" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A72" s="13" t="s">
         <v>442</v>
       </c>
-      <c r="B72" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C72" s="31" t="s">
+      <c r="B72" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C72" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="D72" s="28">
+      <c r="D72" s="25">
         <v>6</v>
       </c>
-      <c r="E72" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F72" s="35" t="s">
+      <c r="E72" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F72" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="G72" s="45">
+      <c r="G72" s="44">
         <v>46112</v>
       </c>
-      <c r="H72" s="31" t="s">
+      <c r="H72" s="13" t="s">
         <v>871</v>
       </c>
-      <c r="I72" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J72" s="31" t="b">
+      <c r="I72" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J72" s="13" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
-      <c r="K72" s="29">
+      <c r="K72" s="21">
         <v>3</v>
       </c>
-      <c r="L72" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="M72" s="27" t="s">
+      <c r="L72" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="M72" s="14" t="s">
         <v>668</v>
       </c>
-      <c r="N72" s="31" t="s">
+      <c r="N72" s="16" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="73" spans="1:14" s="31" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A73" s="31" t="s">
+    <row r="73" spans="1:14" s="13" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A73" s="13" t="s">
         <v>734</v>
       </c>
-      <c r="B73" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C73" s="31" t="s">
+      <c r="B73" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C73" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="D73" s="28">
+      <c r="D73" s="25">
         <v>6</v>
       </c>
-      <c r="E73" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F73" s="35" t="s">
+      <c r="E73" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F73" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="G73" s="45">
+      <c r="G73" s="44">
         <v>46112</v>
       </c>
-      <c r="H73" s="31" t="s">
+      <c r="H73" s="13" t="s">
         <v>871</v>
       </c>
-      <c r="I73" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J73" s="31" t="b">
+      <c r="I73" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J73" s="13" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
-      <c r="K73" s="29">
+      <c r="K73" s="21">
         <v>3</v>
       </c>
-      <c r="L73" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="M73" s="27" t="s">
+      <c r="L73" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="M73" s="14" t="s">
         <v>669</v>
       </c>
-      <c r="N73" s="31" t="s">
+      <c r="N73" s="16" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="74" spans="1:14" s="31" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A74" s="31" t="s">
+    <row r="74" spans="1:14" s="13" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A74" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="B74" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C74" s="31" t="s">
+      <c r="B74" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C74" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="D74" s="28">
+      <c r="D74" s="25">
         <v>6</v>
       </c>
-      <c r="E74" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F74" s="35" t="s">
+      <c r="E74" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F74" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="G74" s="45">
+      <c r="G74" s="44">
         <v>46112</v>
       </c>
-      <c r="H74" s="31" t="s">
+      <c r="H74" s="13" t="s">
         <v>872</v>
       </c>
-      <c r="I74" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J74" s="31" t="b">
+      <c r="I74" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J74" s="13" t="b">
         <f>FALSE</f>
         <v>0</v>
       </c>
-      <c r="K74" s="29"/>
-      <c r="L74" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="M74" s="27" t="s">
+      <c r="K74" s="21"/>
+      <c r="L74" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="M74" s="14" t="s">
         <v>668</v>
       </c>
-      <c r="N74" s="31" t="s">
+      <c r="N74" s="16" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="75" spans="1:14" s="31" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A75" s="31" t="s">
+    <row r="75" spans="1:14" s="13" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A75" s="13" t="s">
         <v>735</v>
       </c>
-      <c r="B75" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C75" s="31" t="s">
+      <c r="B75" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C75" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="D75" s="28">
+      <c r="D75" s="25">
         <v>6</v>
       </c>
-      <c r="E75" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F75" s="35" t="s">
+      <c r="E75" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F75" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="G75" s="45">
+      <c r="G75" s="44">
         <v>46112</v>
       </c>
-      <c r="H75" s="31" t="s">
+      <c r="H75" s="13" t="s">
         <v>872</v>
       </c>
-      <c r="I75" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J75" s="31" t="b">
+      <c r="I75" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J75" s="13" t="b">
         <f>FALSE</f>
         <v>0</v>
       </c>
-      <c r="K75" s="29"/>
-      <c r="L75" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="M75" s="27" t="s">
+      <c r="K75" s="21"/>
+      <c r="L75" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="M75" s="14" t="s">
         <v>669</v>
       </c>
-      <c r="N75" s="31" t="s">
+      <c r="N75" s="16" t="s">
         <v>230</v>
       </c>
     </row>
@@ -11775,91 +11770,91 @@
         <v>536</v>
       </c>
     </row>
-    <row r="214" spans="1:14" s="31" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A214" s="31" t="s">
+    <row r="214" spans="1:14" s="13" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A214" s="38" t="s">
         <v>831</v>
       </c>
-      <c r="B214" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C214" s="31" t="s">
+      <c r="B214" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C214" s="13" t="s">
         <v>545</v>
       </c>
-      <c r="D214" s="28" t="s">
+      <c r="D214" s="25" t="s">
         <v>544</v>
       </c>
-      <c r="E214" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F214" s="35" t="s">
+      <c r="E214" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F214" s="18" t="s">
         <v>825</v>
       </c>
-      <c r="G214" s="42">
+      <c r="G214" s="44">
         <v>46025</v>
       </c>
-      <c r="H214" s="31" t="s">
+      <c r="H214" s="13" t="s">
         <v>845</v>
       </c>
-      <c r="I214" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J214" s="31" t="b">
-        <v>1</v>
-      </c>
-      <c r="K214" s="29">
-        <v>1</v>
-      </c>
-      <c r="L214" s="27" t="s">
+      <c r="I214" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J214" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K214" s="21">
+        <v>1</v>
+      </c>
+      <c r="L214" s="14" t="s">
         <v>827</v>
       </c>
-      <c r="M214" s="27" t="s">
+      <c r="M214" s="14" t="s">
         <v>827</v>
       </c>
-      <c r="N214" s="46" t="s">
+      <c r="N214" s="16" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="215" spans="1:14" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A215" s="31" t="s">
+    <row r="215" spans="1:14" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A215" s="38" t="s">
         <v>832</v>
       </c>
-      <c r="B215" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C215" s="31" t="s">
+      <c r="B215" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C215" s="13" t="s">
         <v>546</v>
       </c>
-      <c r="D215" s="28" t="s">
+      <c r="D215" s="25" t="s">
         <v>544</v>
       </c>
-      <c r="E215" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F215" s="35" t="s">
+      <c r="E215" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F215" s="18" t="s">
         <v>825</v>
       </c>
-      <c r="G215" s="42">
+      <c r="G215" s="44">
         <v>46025</v>
       </c>
-      <c r="H215" s="31" t="s">
+      <c r="H215" s="13" t="s">
         <v>845</v>
       </c>
-      <c r="I215" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J215" s="31" t="b">
-        <v>1</v>
-      </c>
-      <c r="K215" s="29">
-        <v>1</v>
-      </c>
-      <c r="L215" s="27" t="s">
+      <c r="I215" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J215" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K215" s="21">
+        <v>1</v>
+      </c>
+      <c r="L215" s="14" t="s">
         <v>827</v>
       </c>
-      <c r="M215" s="27" t="s">
+      <c r="M215" s="14" t="s">
         <v>827</v>
       </c>
-      <c r="N215" s="46" t="s">
+      <c r="N215" s="16" t="s">
         <v>540</v>
       </c>
     </row>
@@ -11935,7 +11930,7 @@
       <c r="M217" s="4" t="s">
         <v>827</v>
       </c>
-      <c r="N217" s="50" t="s">
+      <c r="N217" s="47" t="s">
         <v>876</v>
       </c>
     </row>
@@ -11973,7 +11968,7 @@
       <c r="M218" s="4" t="s">
         <v>827</v>
       </c>
-      <c r="N218" s="50" t="s">
+      <c r="N218" s="47" t="s">
         <v>877</v>
       </c>
     </row>
@@ -14453,89 +14448,89 @@
         <v>493</v>
       </c>
     </row>
-    <row r="284" spans="1:14" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A284" s="47" t="s">
+    <row r="284" spans="1:14" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A284" s="13" t="s">
         <v>802</v>
       </c>
-      <c r="B284" s="31" t="s">
+      <c r="B284" s="13" t="s">
         <v>563</v>
       </c>
-      <c r="C284" s="48" t="s">
+      <c r="C284" s="13" t="s">
         <v>798</v>
       </c>
-      <c r="D284" s="32" t="s">
+      <c r="D284" s="25" t="s">
         <v>715</v>
       </c>
-      <c r="E284" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F284" s="35" t="s">
+      <c r="E284" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F284" s="39" t="s">
         <v>854</v>
       </c>
-      <c r="G284" s="42">
+      <c r="G284" s="44">
         <v>46112</v>
       </c>
-      <c r="H284" s="31" t="s">
+      <c r="H284" s="13" t="s">
         <v>867</v>
       </c>
-      <c r="I284" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J284" s="31" t="b">
+      <c r="I284" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J284" s="13" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
-      <c r="K284" s="29"/>
-      <c r="L284" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="M284" s="27" t="s">
+      <c r="K284" s="21"/>
+      <c r="L284" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="M284" s="14" t="s">
         <v>800</v>
       </c>
-      <c r="N284" s="31" t="s">
+      <c r="N284" s="13" t="s">
         <v>801</v>
       </c>
     </row>
-    <row r="285" spans="1:14" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A285" s="47" t="s">
+    <row r="285" spans="1:14" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A285" s="13" t="s">
         <v>803</v>
       </c>
-      <c r="B285" s="31" t="s">
+      <c r="B285" s="13" t="s">
         <v>563</v>
       </c>
-      <c r="C285" s="48" t="s">
+      <c r="C285" s="13" t="s">
         <v>799</v>
       </c>
-      <c r="D285" s="32" t="s">
+      <c r="D285" s="25" t="s">
         <v>715</v>
       </c>
-      <c r="E285" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="F285" s="35" t="s">
+      <c r="E285" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="F285" s="39" t="s">
         <v>854</v>
       </c>
-      <c r="G285" s="42">
+      <c r="G285" s="44">
         <v>46112</v>
       </c>
-      <c r="H285" s="31" t="s">
+      <c r="H285" s="13" t="s">
         <v>867</v>
       </c>
-      <c r="I285" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J285" s="31" t="b">
+      <c r="I285" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J285" s="13" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
-      <c r="K285" s="29"/>
-      <c r="L285" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="M285" s="27" t="s">
+      <c r="K285" s="21"/>
+      <c r="L285" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="M285" s="14" t="s">
         <v>800</v>
       </c>
-      <c r="N285" s="31" t="s">
+      <c r="N285" s="13" t="s">
         <v>801</v>
       </c>
     </row>
@@ -15408,7 +15403,7 @@
       <c r="M309" s="4" t="s">
         <v>827</v>
       </c>
-      <c r="N309" s="50" t="s">
+      <c r="N309" s="47" t="s">
         <v>873</v>
       </c>
     </row>
@@ -15446,7 +15441,7 @@
       <c r="M310" s="4" t="s">
         <v>827</v>
       </c>
-      <c r="N310" s="50" t="s">
+      <c r="N310" s="47" t="s">
         <v>874</v>
       </c>
     </row>
@@ -15618,7 +15613,7 @@
       <c r="E315" s="20" t="s">
         <v>345</v>
       </c>
-      <c r="F315" s="49"/>
+      <c r="F315" s="46"/>
       <c r="H315" s="5" t="s">
         <v>869</v>
       </c>

</xml_diff>